<commit_message>
- changed GND of shielding (Ethernet_Port RJ45) - repositioned jumper resistors next to the voltage follower IC - adapted CarrierConnector (changed board height and Connector-Footprint)
</commit_message>
<xml_diff>
--- a/-5V_PCB/PowerManagement_neg5V/Project Outputs for PowerManagement_neg5V/BOM/BOM_PowerManagement_neg5V_1v03.xlsx
+++ b/-5V_PCB/PowerManagement_neg5V/Project Outputs for PowerManagement_neg5V/BOM/BOM_PowerManagement_neg5V_1v03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon\Documents\ultrazohm_analog_ltc2311-16_3vxx\-5V_PCB\PowerManagement_neg5V\Project Outputs for PowerManagement_neg5V\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6FE6FE2F-ACA4-4335-86DA-64CBAFA3F7D4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0DE2C383-63B7-459A-A6FB-790F971FCBAE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="2868" windowWidth="17280" windowHeight="8964" xr2:uid="{D3242623-EECE-49D2-B73D-FE6D11103C18}"/>
+    <workbookView xWindow="2640" yWindow="2868" windowWidth="17280" windowHeight="8964" xr2:uid="{79A4FF15-2505-41C7-B264-5D2FFECB5695}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_PowerManagement_neg5V_1v03" sheetId="1" r:id="rId1"/>
@@ -1101,7 +1101,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A02F2C0A-0CDD-43C0-81D6-ED55DE64F417}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AA7D2E3-66A2-4A52-A3CB-48E5C022E72F}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>